<commit_message>
Update seen store and latest report
</commit_message>
<xml_diff>
--- a/docs/latest.xlsx
+++ b/docs/latest.xlsx
@@ -524,7 +524,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>mobilize:919162:1773599400</t>
+          <t>mobilize:879712:1773514800</t>
         </is>
       </c>
       <c r="D2" t="b">
@@ -532,63 +532,63 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-11T05:39:25</t>
+          <t>2026-03-08T07:16:44</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>RCV Canvass at West Hollywood Meet and Greet for Ankur Patel</t>
+          <t>Tesla Takedown - Stanford Mall</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>11:30 AM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Electric Karma | 8222 1/2 W 3rd St | Los Angeles, CA 90048</t>
+          <t>Tesla Showroom • Stanford Shopping Center | 660 Stanford Shopping Center | Palo Alto, CA 94304</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Beverly Center</t>
+          <t>Stanford Shopping Center</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>BEVCENTER</t>
+          <t>STANFORDSC</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0.43</v>
+        <v>0.02</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://www.mobilize.us/calrcv/event/919162/</t>
+          <t>https://www.mobilize.us/thewolves/event/879712/</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>CANVASS</t>
+          <t>RALLY</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>919162</t>
+          <t>879712</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>1773599400</v>
+        <v>1773514800</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>BEVCENTER:Beverly Center(0.43mi)</t>
+          <t>STANFORDSC:Stanford Shopping Center(0.02mi)</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>mobilize:879712:1773514800</t>
+          <t>mobilize:810382:1773763200</t>
         </is>
       </c>
       <c r="D3" t="b">
@@ -609,63 +609,63 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-08T07:16:44</t>
+          <t>2026-03-11T03:29:59</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Tesla Takedown - Stanford Mall</t>
+          <t>Good Trouble: John Lewis Bridge Overpass! (Northgate) #TeslaTakedownTuesday</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Tesla Showroom • Stanford Shopping Center | 660 Stanford Shopping Center | Palo Alto, CA 94304</t>
+          <t>John Lewis Memorial Bridge Pedestrian Overpass at Northgate | 401 NE Northgate Way | Seattle, WA 98125</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Stanford Shopping Center</t>
+          <t>Northgate Station</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>STANFORDSC</t>
+          <t>NORTHGATE</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://www.mobilize.us/thewolves/event/879712/</t>
+          <t>https://www.mobilize.us/seattleindivisible/event/810382/</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>RALLY</t>
+          <t>VISIBILITY_EVENT</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>879712</t>
+          <t>810382</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>1773514800</v>
+        <v>1773763200</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>STANFORDSC:Stanford Shopping Center(0.02mi)</t>
+          <t>NORTHGATE:Northgate Station(0.2mi)</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>mobilize:810382:1773763200</t>
+          <t>mobilize:810170:1773496800</t>
         </is>
       </c>
       <c r="D4" t="b">
@@ -686,45 +686,45 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-11T03:29:59</t>
+          <t>2026-03-08T07:16:44</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Good Trouble: John Lewis Bridge Overpass! (Northgate) #TeslaTakedownTuesday</t>
+          <t>Visibility CLT Pop-up Protest - Southpark</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>John Lewis Memorial Bridge Pedestrian Overpass at Northgate | 401 NE Northgate Way | Seattle, WA 98125</t>
+          <t>Southpark (Fairview &amp; Sharon) | Fairview Road &amp; Sharon Road | Charlotte, NC 28210</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Northgate Station</t>
+          <t>Southpark</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>NORTHGATE</t>
+          <t>SOUTHPARK</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://www.mobilize.us/seattleindivisible/event/810382/</t>
+          <t>https://www.mobilize.us/indivisiblecharlottenc/event/810170/</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -734,15 +734,15 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>810382</t>
+          <t>810170</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>1773763200</v>
+        <v>1773496800</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NORTHGATE:Northgate Station(0.2mi)</t>
+          <t>SOUTHPARK:Southpark(0.23mi)</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>mobilize:810170:1773496800</t>
+          <t>mobilize:891931:1773597600</t>
         </is>
       </c>
       <c r="D5" t="b">
@@ -763,45 +763,45 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-08T07:16:44</t>
+          <t>2026-03-09T15:27:00</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Visibility CLT Pop-up Protest - Southpark</t>
+          <t>Making Our Resistance Visible</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Southpark (Fairview &amp; Sharon) | Fairview Road &amp; Sharon Road | Charlotte, NC 28210</t>
+          <t>Corner of Green Grove Road and Asbury Avenue in front of the CVS | Tinton Falls, NJ 07753</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Southpark</t>
+          <t>Jersey Shore Premium Outlets</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>SOUTHPARK</t>
+          <t>JERSEYSHOREPO</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.23</v>
+        <v>0.27</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://www.mobilize.us/indivisiblecharlottenc/event/810170/</t>
+          <t>https://www.mobilize.us/indivisible/event/891931/</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -811,15 +811,15 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>810170</t>
+          <t>891931</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>1773496800</v>
+        <v>1773597600</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>SOUTHPARK:Southpark(0.23mi)</t>
+          <t>JERSEYSHOREPO:Jersey Shore Premium Outlets(0.27mi)</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>mobilize:891931:1773597600</t>
+          <t>mobilize:919162:1773599400</t>
         </is>
       </c>
       <c r="D6" t="b">
@@ -840,12 +840,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-03-09T15:27:00</t>
+          <t>2026-03-11T05:39:25</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Making Our Resistance Visible</t>
+          <t>RCV Canvass at West Hollywood Meet and Greet for Ankur Patel</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -855,48 +855,48 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>11:30 AM</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Corner of Green Grove Road and Asbury Avenue in front of the CVS | Tinton Falls, NJ 07753</t>
+          <t>Electric Karma | 8222 1/2 W 3rd St | Los Angeles, CA 90048</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Jersey Shore Premium Outlets</t>
+          <t>Beverly Center</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>JERSEYSHOREPO</t>
+          <t>BEVCENTER</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.27</v>
+        <v>0.43</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://www.mobilize.us/indivisible/event/891931/</t>
+          <t>https://www.mobilize.us/calrcv/event/919162/</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>VISIBILITY_EVENT</t>
+          <t>CANVASS</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>891931</t>
+          <t>919162</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>1773597600</v>
+        <v>1773599400</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>JERSEYSHOREPO:Jersey Shore Premium Outlets(0.27mi)</t>
+          <t>BEVCENTER:Beverly Center(0.43mi)</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:Q59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4874,55 +4874,60 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Last Seen</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Protest Name</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Property ID</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Distance to Property (miles)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Event URL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Event Type</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Event ID</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Timeslot Start (epoch)</t>
         </is>
@@ -4950,53 +4955,58 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>Bridge Brigade over Storrow Drive promoting NO KINGS -March 28</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>4:30 PM</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Appleton Bridge over Storrow Drive to the Esplanade. (Easy access from Red line Charles St station.) | Frances Appleton Brg | Boston, MA 02114</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Copley Place</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>COPLEY</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/bostonindivisible/event/909535/</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>909535</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>1773261000</v>
       </c>
     </row>
@@ -5022,53 +5032,58 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Workshop to Make Art Signs for the Resistance - Boston Indivisible and 50501</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>The Cathedral Church of Saint Paul | 138 Tremont St, Boston | Boston, MA 02111</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Copley Place</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>COPLEY</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.97</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/bostonindivisible/event/909664/</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>WORKSHOP</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>909664</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>1773496800</v>
       </c>
     </row>
@@ -5094,53 +5109,58 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>Brookline Rally for Democracy, March 2026</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>1:00 PM</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Coolidge Corner | Beacon Street &amp; Harvard Street | Brookline, MA 02446</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Copley Place</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>COPLEY</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>2.26</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/speakoutseniors/event/891822/</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>891822</t>
         </is>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>1773507600</v>
       </c>
     </row>
@@ -5166,53 +5186,58 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>Saturday RESIST Standout</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Newton Center | Beacon Street &amp; Centre Street | Newton, MA 02459</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>The Shops at Chestnut Hill</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>CHESTNUTHILL</t>
         </is>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>1.14</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/newtonindivisible/event/892572/</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>892572</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>1773504000</v>
       </c>
     </row>
@@ -5238,53 +5263,58 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>(Panera March 14) Virginia Referendum Postcards</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>2:00 PM</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Panera Bread | 120 Highland Ave | Needham, MA 02494</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>The Shops at Chestnut Hill</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>CHESTNUTHILL</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>2.49</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/swingbluealliance/event/917921/</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>POSTCARD_WRITING</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>917921</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>1773511200</v>
       </c>
     </row>
@@ -5310,53 +5340,58 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>Newton Bridge Brigade—Kendrick St Overpass</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>7:30 AM</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Kendrick Street Overpass | Kendrick St, (Bridge over 128/95) | Needham, MA 02494</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>The Shops at Chestnut Hill</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>CHESTNUTHILL</t>
         </is>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>2.68</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/newtonindivisible/event/897984/</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>897984</t>
         </is>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>1773315000</v>
       </c>
     </row>
@@ -5382,53 +5417,58 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>Needham Resists Visibility Brigade</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>2:45 PM</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Kendrick Street Bridge over 95/128 (park at Cutler Park, 84 Kendrick St) | Kendrick Street | Needham, MA 02494</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>The Shops at Chestnut Hill</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>CHESTNUTHILL</t>
         </is>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>2.68</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/needhamresistsvisibilitybrigade/event/870158/</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>870158</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>1773600300</v>
       </c>
     </row>
@@ -5454,53 +5494,58 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>Highlanders Visibility Brigade—Mass Pike Overpass</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>8:00 AM</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Mass Pike Overpass at Highland St West Newton | Highland St | Newton, MA 02465</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>The Shops at Chestnut Hill</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>CHESTNUTHILL</t>
         </is>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>2.71</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/newtonindivisible/event/898267/</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>898267</t>
         </is>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>1773230400</v>
       </c>
     </row>
@@ -5526,53 +5571,58 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>NO KINGS Protest Airport Rotary Saturday, March 14th 12-1pm</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Airport Rotary | hyannnis, MA 02601</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Cape Cod Mall</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>CAPECOD</t>
         </is>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>0.52</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/899401/</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>899401</t>
         </is>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>1773504000</v>
       </c>
     </row>
@@ -5598,53 +5648,58 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>Exit 4 Nashua Popup Bridge Brigade</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>1:00 PM</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Nashua | Nashua, NH 03062</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Pheasant Lane Mall</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>PHEASANTLANE</t>
         </is>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>2.94</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/nh-bridge-brigade-for-democracy/event/888328/</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>888328</t>
         </is>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>1773594000</v>
       </c>
     </row>
@@ -5670,53 +5725,58 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
           <t>Jersey City KYRs Outreach Walk - South Asian Communities</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Jersey City, NJ 07306</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Newport Centre</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>NEWPORTCTR</t>
         </is>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>1.79</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/aapinewjersey/event/906414/</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>SOLIDARITY_EVENT</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>906414</t>
         </is>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>1773581400</v>
       </c>
     </row>
@@ -5742,53 +5802,58 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>Making Our Resistance Visible</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>2:00 PM</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Corner of Green Grove Road and Asbury Avenue in front of the CVS | Tinton Falls, NJ 07753</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Jersey Shore Premium Outlets</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>JERSEYSHOREPO</t>
         </is>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>0.27</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/891931/</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>891931</t>
         </is>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>1773597600</v>
       </c>
     </row>
@@ -5814,53 +5879,58 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
           <t>Toms River "Hold NJ-CD04 Congressman Chris Smith Accountable" - Protect Democracy</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>33 Washington St | Toms River, NJ 08753</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Ocean County Mall</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>OCEANCOUNTY</t>
         </is>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>2.05</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/900632/</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>900632</t>
         </is>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>1773763200</v>
       </c>
     </row>
@@ -5886,53 +5956,58 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>Signs of Democracy Arlington</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>2:00 PM</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>2710 S Glebe Rd | Arlington, VA 22206</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Fashion Center at Pentagon City</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>PENTAGONCITY</t>
         </is>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>1.59</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/896112/</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>896112</t>
         </is>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>1773511200</v>
       </c>
     </row>
@@ -5958,53 +6033,58 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>WofA Sunday Bridge Brigade</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>2100 21st St N | Arlington, VA 22201</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Fashion Center at Pentagon City</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>PENTAGONCITY</t>
         </is>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>2.7</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/908528/</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>908528</t>
         </is>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>1773601200</v>
       </c>
     </row>
@@ -6030,53 +6110,58 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>Freedom Fridays: Trump, the President of War</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Williamsburg James City County Courthouse | 5201 Monticello Ave | Williamsburg, VA 23188</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Williamsburg Premium Outlets</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>WILLIAMSBURGPO</t>
         </is>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>1.25</v>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/williamsburgjccindivisible/event/918450/</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>918450</t>
         </is>
       </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
         <v>1773417600</v>
       </c>
     </row>
@@ -6102,53 +6187,58 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>Visibility CLT Pop-up Protest - Cotswold</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>4:30 PM</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Randolph &amp; Sharon Amity | Randolph Road &amp; South Sharon Amity Road | Charlotte, NC 28211</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Southpark</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>SOUTHPARK</t>
         </is>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>2.46</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblecharlottenc/event/797821/</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>797821</t>
         </is>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>1773347400</v>
       </c>
     </row>
@@ -6174,53 +6264,58 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
           <t>Visibility CLT Pop-up Protest - Southpark</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Southpark (Fairview &amp; Sharon) | Fairview Road &amp; Sharon Road | Charlotte, NC 28210</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Southpark</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>SOUTHPARK</t>
         </is>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>0.23</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblecharlottenc/event/810170/</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>810170</t>
         </is>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>1773496800</v>
       </c>
     </row>
@@ -6246,53 +6341,58 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>Visibility CLT Pop-up Protest - Park Road Park</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Tyvola Road &amp; Park Road | Charlotte, NC 28210</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Southpark</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>SOUTHPARK</t>
         </is>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>1.03</v>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblecharlottenc/event/816998/</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>816998</t>
         </is>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>1773781200</v>
       </c>
     </row>
@@ -6318,53 +6418,58 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
           <t>Visibility CLT Pop-up Protest - Park Road</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>4:30 PM</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Park Road | Park Road &amp; Woodlawn Road | Charlotte, NC 28209</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Southpark</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>SOUTHPARK</t>
         </is>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>1.82</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblecharlottenc/event/797822/</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>797822</t>
         </is>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>1773347400</v>
       </c>
     </row>
@@ -6390,53 +6495,58 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>Files Into Trials</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>3202 SW 1st Ave | Miami, FL 33145</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>Brickell City Centre</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>BRICKELL</t>
         </is>
       </c>
-      <c r="L22" t="n">
+      <c r="M22" t="n">
         <v>1.71</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/917684/</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>917684</t>
         </is>
       </c>
-      <c r="P22" t="n">
+      <c r="Q22" t="n">
         <v>1773500400</v>
       </c>
     </row>
@@ -6462,53 +6572,58 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
           <t>3/16 South Dade: Community Town Hall</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>6:30 PM</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>11111 Pinkston Dr | Miami, FL 33176</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>The Falls</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>THEFALLS</t>
         </is>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>2.29</v>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/richardforcongress/event/915847/</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>TOWN_HALL</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>915847</t>
         </is>
       </c>
-      <c r="P23" t="n">
+      <c r="Q23" t="n">
         <v>1773700200</v>
       </c>
     </row>
@@ -6534,53 +6649,58 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
           <t>Saturday Sign Waving at Nora Plazas &amp; Monon Trail 11 to 2 PM</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Nora Plazas | East 86th Street &amp; Monon Trail | Indianapolis, IN 46240</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Fashion Mall at Keystone</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>KEYSTONE</t>
         </is>
       </c>
-      <c r="L24" t="n">
+      <c r="M24" t="n">
         <v>1.31</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/hoosiersforconstitutionaldemocracy/event/913681/</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>913681</t>
         </is>
       </c>
-      <c r="P24" t="n">
+      <c r="Q24" t="n">
         <v>1773500400</v>
       </c>
     </row>
@@ -6606,53 +6726,58 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
           <t>No Kings Twin Cities Bridge Brigade -Edina</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Mooty Pickleball Court | 4300 W 66th St | Edina, MN 55435</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Southdale Center</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>SOUTHDALE</t>
         </is>
       </c>
-      <c r="L25" t="n">
+      <c r="M25" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisibletwincities/event/915295/</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="P25" t="inlineStr">
         <is>
           <t>915295</t>
         </is>
       </c>
-      <c r="P25" t="n">
+      <c r="Q25" t="n">
         <v>1773500400</v>
       </c>
     </row>
@@ -6678,53 +6803,58 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
           <t>Anti-ICE Protest at MN GOP HQ (11:30am-12:30pm</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>7400 Metro Blvd | Edina, MN 55439</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Southdale Center</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>SOUTHDALE</t>
         </is>
       </c>
-      <c r="L26" t="n">
+      <c r="M26" t="n">
         <v>1.56</v>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblemn03/event/896393/</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>896393</t>
         </is>
       </c>
-      <c r="P26" t="n">
+      <c r="Q26" t="n">
         <v>1773333000</v>
       </c>
     </row>
@@ -6750,53 +6880,58 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>Rally for Democracy</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>Fulton Neighborhood, Minneapolis | West 50th Street between Upton &amp; Thomas Avenue South, 50th &amp; Upton Avenue South | Minneapolis, MN 55410</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Southdale Center</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>SOUTHDALE</t>
         </is>
       </c>
-      <c r="L27" t="n">
+      <c r="M27" t="n">
         <v>2</v>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/857025/</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>857025</t>
         </is>
       </c>
-      <c r="P27" t="n">
+      <c r="Q27" t="n">
         <v>1773439200</v>
       </c>
     </row>
@@ -6822,53 +6957,58 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
           <t>Rally for Democracy, Stand on Every Corner</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>4:30 PM</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>West 50th Street &amp; Halifax Avenue South | Edina, MN 55424</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Southdale Center</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>SOUTHDALE</t>
         </is>
       </c>
-      <c r="L28" t="n">
+      <c r="M28" t="n">
         <v>2.21</v>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/827822/</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>827822</t>
         </is>
       </c>
-      <c r="P28" t="n">
+      <c r="Q28" t="n">
         <v>1773696600</v>
       </c>
     </row>
@@ -6894,53 +7034,58 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
           <t>Line Colorado Blvd! - Solidarity Saturdays @ 8th Ave</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>8th Avenue &amp; Colorado Boulevard | Denver, CO 80206</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Cherry Creek Shopping Center</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>CHERRYCREEK</t>
         </is>
       </c>
-      <c r="L29" t="n">
+      <c r="M29" t="n">
         <v>1.06</v>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/897610/</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>897610</t>
         </is>
       </c>
-      <c r="P29" t="n">
+      <c r="Q29" t="n">
         <v>1773511200</v>
       </c>
     </row>
@@ -6966,53 +7111,58 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
           <t>Fight Fascism Fridays Vegas</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>Federal Courthouse: Bridger and LVB | 333 S Las Vegas Blvd | Las Vegas, NV 89101</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Las Vegas North Premium Outlets</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>VEGASNORTHPO</t>
         </is>
       </c>
-      <c r="L30" t="n">
+      <c r="M30" t="n">
         <v>0.93</v>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblelasvegas/event/914058/</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>914058</t>
         </is>
       </c>
-      <c r="P30" t="n">
+      <c r="Q30" t="n">
         <v>1773439200</v>
       </c>
     </row>
@@ -7038,53 +7188,58 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>Fight Fascism Fridays Vegas</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>Federal Courthouse: Bridger and LVB | 333 S Las Vegas Blvd | Las Vegas, NV 89101</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>Las Vegas Convention Center</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>VEGASCONVENTION</t>
         </is>
       </c>
-      <c r="L31" t="n">
+      <c r="M31" t="n">
         <v>2.38</v>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblelasvegas/event/914058/</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>914058</t>
         </is>
       </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
         <v>1773439200</v>
       </c>
     </row>
@@ -7110,53 +7265,58 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
           <t>Fight Fascism Fridays Vegas</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>Federal Courthouse: Bridger and LVB | 333 S Las Vegas Blvd | Las Vegas, NV 89101</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>Encore at Wynn Las Vegas</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>ENCOREWYNNVEGAS</t>
         </is>
       </c>
-      <c r="L32" t="n">
+      <c r="M32" t="n">
         <v>2.78</v>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblelasvegas/event/914058/</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>914058</t>
         </is>
       </c>
-      <c r="P32" t="n">
+      <c r="Q32" t="n">
         <v>1773439200</v>
       </c>
     </row>
@@ -7173,7 +7333,7 @@
         </is>
       </c>
       <c r="D33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7182,53 +7342,58 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
           <t>RCV Canvass at West Hollywood Meet and Greet for Ankur Patel</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>Electric Karma | 8222 1/2 W 3rd St | Los Angeles, CA 90048</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>Beverly Center</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>BEVCENTER</t>
         </is>
       </c>
-      <c r="L33" t="n">
+      <c r="M33" t="n">
         <v>0.43</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/calrcv/event/919162/</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>CANVASS</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="P33" t="inlineStr">
         <is>
           <t>919162</t>
         </is>
       </c>
-      <c r="P33" t="n">
+      <c r="Q33" t="n">
         <v>1773599400</v>
       </c>
     </row>
@@ -7254,53 +7419,58 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
           <t>Liberty and Justice for ALL, South Bay</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>Northeast corner Anza at PCH | 4135 Pacific Coast Hwy | Torrance, CA 90505</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>Del Amo Fashion Center</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>DELAMO</t>
         </is>
       </c>
-      <c r="L34" t="n">
+      <c r="M34" t="n">
         <v>1.66</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblesouthbayla/event/916557/</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>916557</t>
         </is>
       </c>
-      <c r="P34" t="n">
+      <c r="Q34" t="n">
         <v>1773513000</v>
       </c>
     </row>
@@ -7326,53 +7496,58 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
           <t>Fight Fascism Fridays - Every Friday in Rancho Cucamonga</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>Haven Avenue &amp; Foothill Boulevard | Rancho Cucamonga, CA 91730</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>Ontario Mills</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>ONTARIOMILLS</t>
         </is>
       </c>
-      <c r="L35" t="n">
+      <c r="M35" t="n">
         <v>2.81</v>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/catladiesforamerica/event/893656/</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>893656</t>
         </is>
       </c>
-      <c r="P35" t="n">
+      <c r="Q35" t="n">
         <v>1773441000</v>
       </c>
     </row>
@@ -7398,53 +7573,58 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
           <t>Weekly Meade Ave Bridge Bannering Over I-805 | Thursday Afternoons</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>Meade Ave Bridge Over I-805 | 4371 Boundary St | San Diego, CA 92116</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>Fashion Valley</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>FASHIONVAL</t>
         </is>
       </c>
-      <c r="L36" t="n">
+      <c r="M36" t="n">
         <v>2.41</v>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/visibilitybrigadesandiego/event/860202/</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="P36" t="inlineStr">
         <is>
           <t>860202</t>
         </is>
       </c>
-      <c r="P36" t="n">
+      <c r="Q36" t="n">
         <v>1773360000</v>
       </c>
     </row>
@@ -7470,53 +7650,58 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
           <t>Visibility Brigade - North Park</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>Meade Ave bridge over I-805 in North Park | 4371 Boundary St | San Diego, CA 92116</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>Fashion Valley</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>FASHIONVAL</t>
         </is>
       </c>
-      <c r="L37" t="n">
+      <c r="M37" t="n">
         <v>2.41</v>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/824060/</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="P37" t="inlineStr">
         <is>
           <t>824060</t>
         </is>
       </c>
-      <c r="P37" t="n">
+      <c r="Q37" t="n">
         <v>1773360000</v>
       </c>
     </row>
@@ -7542,53 +7727,58 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
           <t>Weekly Taylor St Bridge Bannering Over I-8 | Monday Afternoons</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>4:00 PM</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>Taylor Street Bridge (Exit 3) | 4490 Taylor St, Taylor Street Park and Ride | San Diego, CA 92108</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>Fashion Valley</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>FASHIONVAL</t>
         </is>
       </c>
-      <c r="L38" t="n">
+      <c r="M38" t="n">
         <v>1.54</v>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/visibilitybrigadesandiego/event/871084/</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="P38" t="inlineStr">
         <is>
           <t>871084</t>
         </is>
       </c>
-      <c r="P38" t="n">
+      <c r="Q38" t="n">
         <v>1773702000</v>
       </c>
     </row>
@@ -7614,53 +7804,58 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
           <t>Weekly Taylor St Bridge Bannering Over I-8 | Monday Afternoons - Visibility Brigade</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>4:00 PM</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>Taylor Street Bridge (Exit 3) | 4490 Taylor St, Taylor Street Park and Ride | San Diego, CA 92108</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Fashion Valley</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>FASHIONVAL</t>
         </is>
       </c>
-      <c r="L39" t="n">
+      <c r="M39" t="n">
         <v>1.54</v>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/875118/</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="P39" t="inlineStr">
         <is>
           <t>875118</t>
         </is>
       </c>
-      <c r="P39" t="n">
+      <c r="Q39" t="n">
         <v>1773702000</v>
       </c>
     </row>
@@ -7686,53 +7881,58 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
           <t>Change Begins With ME Overpass Alliance-Mondays</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>4:00 PM</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>Clairemont Drive overpass at I-5 | 2366 Clairemont Dr | San Diego, CA 92109</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>Fashion Valley</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>FASHIONVAL</t>
         </is>
       </c>
-      <c r="L40" t="n">
+      <c r="M40" t="n">
         <v>2.87</v>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/bethechangesd/event/824571/</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
+      <c r="P40" t="inlineStr">
         <is>
           <t>824571</t>
         </is>
       </c>
-      <c r="P40" t="n">
+      <c r="Q40" t="n">
         <v>1773702000</v>
       </c>
     </row>
@@ -7758,53 +7958,58 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
           <t>Say No To Ken Calvert Weekly Visibility Sign Waving- Formerly Empty Chair Town Hall!</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>Intersection of Monterrey and 111- park at Panera | 73075 CA-111 | Palm Desert, CA 92260</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>The Gardens on El Paseo</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>GARDENSONELPASO</t>
         </is>
       </c>
-      <c r="L41" t="n">
+      <c r="M41" t="n">
         <v>0.52</v>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/801600/</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="P41" t="inlineStr">
         <is>
           <t>801600</t>
         </is>
       </c>
-      <c r="P41" t="n">
+      <c r="Q41" t="n">
         <v>1773590400</v>
       </c>
     </row>
@@ -7830,53 +8035,58 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>Defend Democracy. Demand Accountability.</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>La Paz Road &amp; Marguerite Parkway | Mission Viejo, CA 92692</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>The Shops at Mission Viejo</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>MISSIONVIEJO</t>
         </is>
       </c>
-      <c r="L42" t="n">
+      <c r="M42" t="n">
         <v>2.71</v>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisibleca40/event/823056/</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="P42" t="inlineStr">
         <is>
           <t>823056</t>
         </is>
       </c>
-      <c r="P42" t="n">
+      <c r="Q42" t="n">
         <v>1773252000</v>
       </c>
     </row>
@@ -7902,53 +8112,58 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>Ladera Ranch Stands For Human Rights</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Crown Valley &amp; Antonio | 27402 Antonio Pkwy | Ladera Ranch, CA 92694</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>The Shops at Mission Viejo</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>MISSIONVIEJO</t>
         </is>
       </c>
-      <c r="L43" t="n">
+      <c r="M43" t="n">
         <v>2.39</v>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/ocindivisible/event/893284/</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>893284</t>
         </is>
       </c>
-      <c r="P43" t="n">
+      <c r="Q43" t="n">
         <v>1773446400</v>
       </c>
     </row>
@@ -7974,53 +8189,58 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
           <t>Overpass Brigade</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>4:30 PM</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>East Grand Avenue overpass near The Village | E Grand Ave &amp; Hwy. 101 | Arroyo Grande, CA 93420</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>Pismo Beach Premium Outlets</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>PISMOBEACH</t>
         </is>
       </c>
-      <c r="L44" t="n">
+      <c r="M44" t="n">
         <v>2.7</v>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/917108/</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="O44" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="P44" t="inlineStr">
         <is>
           <t>917108</t>
         </is>
       </c>
-      <c r="P44" t="n">
+      <c r="Q44" t="n">
         <v>1773444600</v>
       </c>
     </row>
@@ -8046,53 +8266,58 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
           <t>Signs of Fascism (Palo Alto)</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>Corner of El Camino Real and Embarcadero Road | 50 Embarcadero Rd | Palo Alto, CA 94301</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>Stanford Shopping Center</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>STANFORDSC</t>
         </is>
       </c>
-      <c r="L45" t="n">
+      <c r="M45" t="n">
         <v>0.84</v>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/ipaplus/event/876104/</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="P45" t="inlineStr">
         <is>
           <t>876104</t>
         </is>
       </c>
-      <c r="P45" t="n">
+      <c r="Q45" t="n">
         <v>1773426600</v>
       </c>
     </row>
@@ -8118,53 +8343,58 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
           <t>Tesla Takedown - Stanford Mall</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>Tesla Showroom • Stanford Shopping Center | 660 Stanford Shopping Center | Palo Alto, CA 94304</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>Stanford Shopping Center</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>STANFORDSC</t>
         </is>
       </c>
-      <c r="L46" t="n">
+      <c r="M46" t="n">
         <v>0.02</v>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/thewolves/event/879712/</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="O46" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="P46" t="inlineStr">
         <is>
           <t>879712</t>
         </is>
       </c>
-      <c r="P46" t="n">
+      <c r="Q46" t="n">
         <v>1773514800</v>
       </c>
     </row>
@@ -8190,53 +8420,58 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
           <t>Union Busting Billionaires Gotta Go!</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>Whole Foods Market | 774 Emerson St | Palo Alto, CA 94301</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>Stanford Shopping Center</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>STANFORDSC</t>
         </is>
       </c>
-      <c r="L47" t="n">
+      <c r="M47" t="n">
         <v>0.63</v>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/thewolves/event/875874/</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
+      <c r="O47" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>875874</t>
         </is>
       </c>
-      <c r="P47" t="n">
+      <c r="Q47" t="n">
         <v>1773705600</v>
       </c>
     </row>
@@ -8262,53 +8497,58 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
           <t>Menlo Park Speaks Out</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>10:30 AM</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>Fremont Park | University Drive &amp; Santa Cruz Avenue | Menlo Park, CA 94025</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Stanford Shopping Center</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>STANFORDSC</t>
         </is>
       </c>
-      <c r="L48" t="n">
+      <c r="M48" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="N48" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/menloparkspeaksout/event/791569/</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="O48" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>791569</t>
         </is>
       </c>
-      <c r="P48" t="n">
+      <c r="Q48" t="n">
         <v>1773595800</v>
       </c>
     </row>
@@ -8334,53 +8574,58 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
           <t>Bannering 101 (Palo Alto)</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>Adobe Creek Bike and Pedestrian Bridge | Palo Alto, CA 94303</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>Stanford Shopping Center</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>STANFORDSC</t>
         </is>
       </c>
-      <c r="L49" t="n">
+      <c r="M49" t="n">
         <v>3</v>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="N49" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/ipaplus/event/836661/</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
+      <c r="O49" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
+      <c r="P49" t="inlineStr">
         <is>
           <t>836661</t>
         </is>
       </c>
-      <c r="P49" t="n">
+      <c r="Q49" t="n">
         <v>1773248400</v>
       </c>
     </row>
@@ -8406,53 +8651,58 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
           <t>Weekly Napa Rally to Resist the Trump/Musk/GOP Regime!</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>Soscol Avenue &amp; 3rd Street | Napa, CA 94559</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>Napa Premium Outlets</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>NAPAPO</t>
         </is>
       </c>
-      <c r="L50" t="n">
+      <c r="M50" t="n">
         <v>1.14</v>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="N50" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisible/event/774947/</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="P50" t="inlineStr">
         <is>
           <t>774947</t>
         </is>
       </c>
-      <c r="P50" t="n">
+      <c r="Q50" t="n">
         <v>1773446400</v>
       </c>
     </row>
@@ -8478,53 +8728,58 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
           <t>Justice for Renée Good / Alex Pretti - ICE out of Home Depot Protest</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>Bicentennial Way &amp; Mendocino Avenue | Santa Rosa, CA 95403</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>Santa Rosa Plaza</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>SANTAROSA</t>
         </is>
       </c>
-      <c r="L51" t="n">
+      <c r="M51" t="n">
         <v>2.2</v>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="N51" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblesonomacounty/event/838660/</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
+      <c r="O51" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr">
+      <c r="P51" t="inlineStr">
         <is>
           <t>838660</t>
         </is>
       </c>
-      <c r="P51" t="n">
+      <c r="Q51" t="n">
         <v>1773597600</v>
       </c>
     </row>
@@ -8550,53 +8805,58 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
           <t>VISIBILITY BRIGADE - Santa Rosa - 101 Ped Bridge @ Hwy 12</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>Santa Rosa Pedestrian Overpass, over Hwy 101 and just south of Hwy 12. Access to the "sky bridge" using your mobile map app. | 808 S. Davis St., 935 S. A. St. | Santa Rosa, CA 95407</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>Santa Rosa Plaza</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>SANTAROSA</t>
         </is>
       </c>
-      <c r="L52" t="n">
+      <c r="M52" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="N52" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblesonomacounty/event/795435/</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="O52" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
+      <c r="P52" t="inlineStr">
         <is>
           <t>795435</t>
         </is>
       </c>
-      <c r="P52" t="n">
+      <c r="Q52" t="n">
         <v>1773268200</v>
       </c>
     </row>
@@ -8622,53 +8882,58 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
           <t>Tell Target: ICE OUT NOW - Justice for Renee Good &amp; Alex Pretti</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>Target - Santa Rosa South (public sidewalks) | 1980 Santa Rosa Ave, (Meet at the Kawana Springs Rd. driveway entrance to Target Shopping center (traffic signal) | Santa Rosa, CA 95404</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>Santa Rosa Plaza</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="L53" t="inlineStr">
         <is>
           <t>SANTAROSA</t>
         </is>
       </c>
-      <c r="L53" t="n">
+      <c r="M53" t="n">
         <v>1.55</v>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="N53" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/indivisiblesonomacounty/event/848553/</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="O53" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
+      <c r="P53" t="inlineStr">
         <is>
           <t>848553</t>
         </is>
       </c>
-      <c r="P53" t="n">
+      <c r="Q53" t="n">
         <v>1773511200</v>
       </c>
     </row>
@@ -8694,53 +8959,58 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
           <t>CRUSH ICE! NO SECRET POLICE! WEEKLY THURSDAYS!! (Honolulu)</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>Intersection of Atkinson Drive &amp; Ala Moana Boulevard | Atkinson Drive &amp; Ala Moana Boulevard | Honolulu, HI 96814</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>International Market Place</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>INTLMARKET</t>
         </is>
       </c>
-      <c r="L54" t="n">
+      <c r="M54" t="n">
         <v>1.25</v>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="N54" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/protecthawaii/event/826166/</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
+      <c r="O54" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
+      <c r="P54" t="inlineStr">
         <is>
           <t>826166</t>
         </is>
       </c>
-      <c r="P54" t="n">
+      <c r="Q54" t="n">
         <v>1773370800</v>
       </c>
     </row>
@@ -8766,53 +9036,58 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
           <t>Good Trouble: John Lewis Bridge Overpass! (Northgate) #TeslaTakedownTuesday</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="H55" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>John Lewis Memorial Bridge Pedestrian Overpass at Northgate | 401 NE Northgate Way | Seattle, WA 98125</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>Northgate Station</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>NORTHGATE</t>
         </is>
       </c>
-      <c r="L55" t="n">
+      <c r="M55" t="n">
         <v>0.2</v>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/seattleindivisible/event/810382/</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
+      <c r="O55" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr">
+      <c r="P55" t="inlineStr">
         <is>
           <t>810382</t>
         </is>
       </c>
-      <c r="P55" t="n">
+      <c r="Q55" t="n">
         <v>1773763200</v>
       </c>
     </row>
@@ -8838,53 +9113,58 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
           <t>Tesla Takedown Tuesday: Woodland Park Overpass!</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>4:00 PM</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>Woodland Park N Pedestrian Bridge | 5192 Aurora Ave N | Seattle, WA 98103</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>Northgate Station</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="L56" t="inlineStr">
         <is>
           <t>NORTHGATE</t>
         </is>
       </c>
-      <c r="L56" t="n">
+      <c r="M56" t="n">
         <v>2.81</v>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="N56" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/seattleindivisible/event/807188/</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
+      <c r="O56" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr">
+      <c r="P56" t="inlineStr">
         <is>
           <t>807188</t>
         </is>
       </c>
-      <c r="P56" t="n">
+      <c r="Q56" t="n">
         <v>1773788400</v>
       </c>
     </row>
@@ -8910,53 +9190,58 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
           <t>Refuse Fascism Fridays-Marysville (Other locations, see Details)</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>Fourth Street &amp; State Avenue | Marysville, WA 98270</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>Seattle Premium Outlets</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="L57" t="inlineStr">
         <is>
           <t>SEATTLEPO</t>
         </is>
       </c>
-      <c r="L57" t="n">
+      <c r="M57" t="n">
         <v>2.88</v>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/snohomishcountyindivisible/event/899741/</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
+      <c r="O57" t="inlineStr">
         <is>
           <t>RALLY</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr">
+      <c r="P57" t="inlineStr">
         <is>
           <t>899741</t>
         </is>
       </c>
-      <c r="P57" t="n">
+      <c r="Q57" t="n">
         <v>1773446400</v>
       </c>
     </row>
@@ -8982,53 +9267,58 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
           <t>NO WAR. NO KINGS: Tacoma</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="J58" t="inlineStr">
         <is>
           <t>Union Station - Federal Courthouse | 1717 Pacific Ave | Tacoma, WA 98402</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>Tacoma Mall</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
+      <c r="L58" t="inlineStr">
         <is>
           <t>TACOMAMALL</t>
         </is>
       </c>
-      <c r="L58" t="n">
+      <c r="M58" t="n">
         <v>2.59</v>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="N58" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/seattleindivisible/event/795854/</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
+      <c r="O58" t="inlineStr">
         <is>
           <t>VISIBILITY_EVENT</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr">
+      <c r="P58" t="inlineStr">
         <is>
           <t>795854</t>
         </is>
       </c>
-      <c r="P58" t="n">
+      <c r="Q58" t="n">
         <v>1773507600</v>
       </c>
     </row>
@@ -9054,58 +9344,63 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
+          <t>2026-03-11T06:33:53</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
           <t>Knock doors with Team Sydney for Assembly!</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="J59" t="inlineStr">
         <is>
           <t>Location provided upon RSVP | Throughout North Anchorage! | Anchorage, AK 99501</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t>Anchorage 5th Avenue Mall</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="L59" t="inlineStr">
         <is>
           <t>ANC5Ave</t>
         </is>
       </c>
-      <c r="L59" t="n">
+      <c r="M59" t="n">
         <v>0.73</v>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="N59" t="inlineStr">
         <is>
           <t>https://www.mobilize.us/sydneyscoutforassembly/event/918417/</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
+      <c r="O59" t="inlineStr">
         <is>
           <t>CANVASS</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr">
+      <c r="P59" t="inlineStr">
         <is>
           <t>918417</t>
         </is>
       </c>
-      <c r="P59" t="n">
+      <c r="Q59" t="n">
         <v>1773604800</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:P59">
+  <conditionalFormatting sqref="A2:Q59">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D2=TRUE</formula>
     </cfRule>

</xml_diff>